<commit_message>
All images reviewed and approved
</commit_message>
<xml_diff>
--- a/work/drawing_svg_review/Review_result.xlsx
+++ b/work/drawing_svg_review/Review_result.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\jjcarron\proj\50ohm\ham-translator\50ohm-contents-ch\work\drawing_svg_review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21C8C70E-F498-42C6-8430-D9299C6E1378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F80771BC-BED2-471E-A0C9-B4F33197EF99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26190" yWindow="3000" windowWidth="32820" windowHeight="15945" xr2:uid="{5DFD519D-02CF-4758-86F1-0D550B48092E}"/>
+    <workbookView xWindow="-27915" yWindow="4110" windowWidth="26055" windowHeight="15945" xr2:uid="{5DFD519D-02CF-4758-86F1-0D550B48092E}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="180">
   <si>
     <t>1000.de.svg</t>
   </si>
@@ -579,72 +579,6 @@
   </si>
   <si>
     <t>Ok</t>
-  </si>
-  <si>
-    <t>Not translated</t>
-  </si>
-  <si>
-    <t>PDF copy</t>
-  </si>
-  <si>
-    <t>partially translated</t>
-  </si>
-  <si>
-    <t>MWS non traduis</t>
-  </si>
-  <si>
-    <t>Traduction à corriger</t>
-  </si>
-  <si>
-    <t>Traduction à corriger N/A-&gt; D/A</t>
-  </si>
-  <si>
-    <t>Traduction à corriger de gain</t>
-  </si>
-  <si>
-    <t>Taille du texte non respectée</t>
-  </si>
-  <si>
-    <t>other</t>
-  </si>
-  <si>
-    <t>HF-Diode = Diode HF</t>
-  </si>
-  <si>
-    <t>Commande etsignaus de contrôle</t>
-  </si>
-  <si>
-    <t>emplacement -&gt; position</t>
-  </si>
-  <si>
-    <t>texte trop long sur une ligne mettre sur deux lignes</t>
-  </si>
-  <si>
-    <t>Superposition de txte (non suppression de l'allemand?</t>
-  </si>
-  <si>
-    <t>Voltmètre</t>
-  </si>
-  <si>
-    <t>FZD -&gt; FFI et FIF</t>
-  </si>
-  <si>
-    <t>ZF et NF</t>
-  </si>
-  <si>
-    <t>Eingangsignal, Verstärkung, ausgangsignal</t>
-  </si>
-  <si>
-    <t>MWS not translated</t>
-  </si>
-  <si>
-    <t>Voltmetre</t>
-  </si>
-  <si>
-    <t>ampèremètre</t>
-  </si>
-  <si>
-    <t>Phys. Stromrichtung</t>
   </si>
 </sst>
 </file>
@@ -1065,7 +999,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
-        <f>--_xlfn.TEXTBEFORE(B2,".")</f>
+        <f t="shared" ref="A2:A33" si="0">--_xlfn.TEXTBEFORE(B2,".")</f>
         <v>44</v>
       </c>
       <c r="B2" t="s">
@@ -1080,7 +1014,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
-        <f>--_xlfn.TEXTBEFORE(B3,".")</f>
+        <f t="shared" si="0"/>
         <v>45</v>
       </c>
       <c r="B3" t="s">
@@ -1095,7 +1029,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
-        <f>--_xlfn.TEXTBEFORE(B4,".")</f>
+        <f t="shared" si="0"/>
         <v>46</v>
       </c>
       <c r="B4" t="s">
@@ -1110,7 +1044,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
-        <f>--_xlfn.TEXTBEFORE(B5,".")</f>
+        <f t="shared" si="0"/>
         <v>49</v>
       </c>
       <c r="B5" t="s">
@@ -1125,7 +1059,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
-        <f>--_xlfn.TEXTBEFORE(B6,".")</f>
+        <f t="shared" si="0"/>
         <v>65</v>
       </c>
       <c r="B6" t="s">
@@ -1140,7 +1074,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
-        <f>--_xlfn.TEXTBEFORE(B7,".")</f>
+        <f t="shared" si="0"/>
         <v>80</v>
       </c>
       <c r="B7" t="s">
@@ -1155,7 +1089,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
-        <f>--_xlfn.TEXTBEFORE(B8,".")</f>
+        <f t="shared" si="0"/>
         <v>85</v>
       </c>
       <c r="B8" t="s">
@@ -1170,7 +1104,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
-        <f>--_xlfn.TEXTBEFORE(B9,".")</f>
+        <f t="shared" si="0"/>
         <v>86</v>
       </c>
       <c r="B9" t="s">
@@ -1185,7 +1119,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
-        <f>--_xlfn.TEXTBEFORE(B10,".")</f>
+        <f t="shared" si="0"/>
         <v>96</v>
       </c>
       <c r="B10" t="s">
@@ -1200,7 +1134,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
-        <f>--_xlfn.TEXTBEFORE(B11,".")</f>
+        <f t="shared" si="0"/>
         <v>98</v>
       </c>
       <c r="B11" t="s">
@@ -1215,7 +1149,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
-        <f>--_xlfn.TEXTBEFORE(B12,".")</f>
+        <f t="shared" si="0"/>
         <v>105</v>
       </c>
       <c r="B12" t="s">
@@ -1230,7 +1164,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
-        <f>--_xlfn.TEXTBEFORE(B13,".")</f>
+        <f t="shared" si="0"/>
         <v>141</v>
       </c>
       <c r="B13" t="s">
@@ -1245,7 +1179,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
-        <f>--_xlfn.TEXTBEFORE(B14,".")</f>
+        <f t="shared" si="0"/>
         <v>142</v>
       </c>
       <c r="B14" t="s">
@@ -1260,7 +1194,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
-        <f>--_xlfn.TEXTBEFORE(B15,".")</f>
+        <f t="shared" si="0"/>
         <v>149</v>
       </c>
       <c r="B15" t="s">
@@ -1275,7 +1209,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
-        <f>--_xlfn.TEXTBEFORE(B16,".")</f>
+        <f t="shared" si="0"/>
         <v>153</v>
       </c>
       <c r="B16" t="s">
@@ -1288,9 +1222,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
-        <f>--_xlfn.TEXTBEFORE(B17,".")</f>
+        <f t="shared" si="0"/>
         <v>155</v>
       </c>
       <c r="B17" t="s">
@@ -1303,9 +1237,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
-        <f>--_xlfn.TEXTBEFORE(B18,".")</f>
+        <f t="shared" si="0"/>
         <v>158</v>
       </c>
       <c r="B18" t="s">
@@ -1318,27 +1252,24 @@
         <v>179</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
-        <f>--_xlfn.TEXTBEFORE(B19,".")</f>
+        <f t="shared" si="0"/>
         <v>202</v>
       </c>
       <c r="B19" t="s">
         <v>39</v>
       </c>
       <c r="C19" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D19" t="s">
-        <v>180</v>
-      </c>
-      <c r="E19" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
-        <f>--_xlfn.TEXTBEFORE(B20,".")</f>
+        <f t="shared" si="0"/>
         <v>250</v>
       </c>
       <c r="B20" t="s">
@@ -1351,9 +1282,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
-        <f>--_xlfn.TEXTBEFORE(B21,".")</f>
+        <f t="shared" si="0"/>
         <v>251</v>
       </c>
       <c r="B21" t="s">
@@ -1366,9 +1297,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
-        <f>--_xlfn.TEXTBEFORE(B22,".")</f>
+        <f t="shared" si="0"/>
         <v>252</v>
       </c>
       <c r="B22" t="s">
@@ -1381,9 +1312,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
-        <f>--_xlfn.TEXTBEFORE(B23,".")</f>
+        <f t="shared" si="0"/>
         <v>253</v>
       </c>
       <c r="B23" t="s">
@@ -1396,9 +1327,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
-        <f>--_xlfn.TEXTBEFORE(B24,".")</f>
+        <f t="shared" si="0"/>
         <v>258</v>
       </c>
       <c r="B24" t="s">
@@ -1411,9 +1342,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
-        <f>--_xlfn.TEXTBEFORE(B25,".")</f>
+        <f t="shared" si="0"/>
         <v>259</v>
       </c>
       <c r="B25" t="s">
@@ -1426,27 +1357,24 @@
         <v>179</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26">
-        <f>--_xlfn.TEXTBEFORE(B26,".")</f>
+        <f t="shared" si="0"/>
         <v>260</v>
       </c>
       <c r="B26" t="s">
         <v>46</v>
       </c>
       <c r="C26" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D26" t="s">
-        <v>182</v>
-      </c>
-      <c r="E26" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27">
-        <f>--_xlfn.TEXTBEFORE(B27,".")</f>
+        <f t="shared" si="0"/>
         <v>264</v>
       </c>
       <c r="B27" t="s">
@@ -1459,9 +1387,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28">
-        <f>--_xlfn.TEXTBEFORE(B28,".")</f>
+        <f t="shared" si="0"/>
         <v>303</v>
       </c>
       <c r="B28" t="s">
@@ -1474,9 +1402,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29">
-        <f>--_xlfn.TEXTBEFORE(B29,".")</f>
+        <f t="shared" si="0"/>
         <v>311</v>
       </c>
       <c r="B29" t="s">
@@ -1489,27 +1417,24 @@
         <v>179</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30">
-        <f>--_xlfn.TEXTBEFORE(B30,".")</f>
+        <f t="shared" si="0"/>
         <v>315</v>
       </c>
       <c r="B30" t="s">
         <v>50</v>
       </c>
       <c r="C30" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D30" t="s">
-        <v>182</v>
-      </c>
-      <c r="E30" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31">
-        <f>--_xlfn.TEXTBEFORE(B31,".")</f>
+        <f t="shared" si="0"/>
         <v>341</v>
       </c>
       <c r="B31" t="s">
@@ -1522,9 +1447,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32">
-        <f>--_xlfn.TEXTBEFORE(B32,".")</f>
+        <f t="shared" si="0"/>
         <v>342</v>
       </c>
       <c r="B32" t="s">
@@ -1537,9 +1462,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33">
-        <f>--_xlfn.TEXTBEFORE(B33,".")</f>
+        <f t="shared" si="0"/>
         <v>354</v>
       </c>
       <c r="B33" t="s">
@@ -1552,9 +1477,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34">
-        <f>--_xlfn.TEXTBEFORE(B34,".")</f>
+        <f t="shared" ref="A34:A65" si="1">--_xlfn.TEXTBEFORE(B34,".")</f>
         <v>355</v>
       </c>
       <c r="B34" t="s">
@@ -1567,9 +1492,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35">
-        <f>--_xlfn.TEXTBEFORE(B35,".")</f>
+        <f t="shared" si="1"/>
         <v>423</v>
       </c>
       <c r="B35" t="s">
@@ -1582,9 +1507,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36">
-        <f>--_xlfn.TEXTBEFORE(B36,".")</f>
+        <f t="shared" si="1"/>
         <v>424</v>
       </c>
       <c r="B36" t="s">
@@ -1597,9 +1522,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37">
-        <f>--_xlfn.TEXTBEFORE(B37,".")</f>
+        <f t="shared" si="1"/>
         <v>430</v>
       </c>
       <c r="B37" t="s">
@@ -1612,45 +1537,39 @@
         <v>179</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38">
-        <f>--_xlfn.TEXTBEFORE(B38,".")</f>
+        <f t="shared" si="1"/>
         <v>434</v>
       </c>
       <c r="B38" t="s">
         <v>58</v>
       </c>
       <c r="C38" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D38" t="s">
-        <v>182</v>
-      </c>
-      <c r="E38" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39">
-        <f>--_xlfn.TEXTBEFORE(B39,".")</f>
+        <f t="shared" si="1"/>
         <v>435</v>
       </c>
       <c r="B39" t="s">
         <v>59</v>
       </c>
       <c r="C39" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D39" t="s">
-        <v>182</v>
-      </c>
-      <c r="E39" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40">
-        <f>--_xlfn.TEXTBEFORE(B40,".")</f>
+        <f t="shared" si="1"/>
         <v>436</v>
       </c>
       <c r="B40" t="s">
@@ -1663,9 +1582,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41">
-        <f>--_xlfn.TEXTBEFORE(B41,".")</f>
+        <f t="shared" si="1"/>
         <v>437</v>
       </c>
       <c r="B41" t="s">
@@ -1678,45 +1597,39 @@
         <v>179</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42">
-        <f>--_xlfn.TEXTBEFORE(B42,".")</f>
+        <f t="shared" si="1"/>
         <v>438</v>
       </c>
       <c r="B42" t="s">
         <v>62</v>
       </c>
       <c r="C42" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D42" t="s">
-        <v>182</v>
-      </c>
-      <c r="E42" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43">
-        <f>--_xlfn.TEXTBEFORE(B43,".")</f>
+        <f t="shared" si="1"/>
         <v>439</v>
       </c>
       <c r="B43" t="s">
         <v>63</v>
       </c>
       <c r="C43" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D43" t="s">
-        <v>182</v>
-      </c>
-      <c r="E43" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44">
-        <f>--_xlfn.TEXTBEFORE(B44,".")</f>
+        <f t="shared" si="1"/>
         <v>443</v>
       </c>
       <c r="B44" t="s">
@@ -1729,27 +1642,24 @@
         <v>179</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45">
-        <f>--_xlfn.TEXTBEFORE(B45,".")</f>
+        <f t="shared" si="1"/>
         <v>471</v>
       </c>
       <c r="B45" t="s">
         <v>68</v>
       </c>
       <c r="C45" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="D45" t="s">
-        <v>188</v>
-      </c>
-      <c r="E45" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46">
-        <f>--_xlfn.TEXTBEFORE(B46,".")</f>
+        <f t="shared" si="1"/>
         <v>475</v>
       </c>
       <c r="B46" t="s">
@@ -1762,45 +1672,39 @@
         <v>179</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47">
-        <f>--_xlfn.TEXTBEFORE(B47,".")</f>
+        <f t="shared" si="1"/>
         <v>496</v>
       </c>
       <c r="B47" t="s">
         <v>71</v>
       </c>
       <c r="C47" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D47" t="s">
-        <v>182</v>
-      </c>
-      <c r="E47" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48">
-        <f>--_xlfn.TEXTBEFORE(B48,".")</f>
+        <f t="shared" si="1"/>
         <v>501</v>
       </c>
       <c r="B48" t="s">
         <v>72</v>
       </c>
       <c r="C48" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D48" t="s">
-        <v>182</v>
-      </c>
-      <c r="E48" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49">
-        <f>--_xlfn.TEXTBEFORE(B49,".")</f>
+        <f t="shared" si="1"/>
         <v>590</v>
       </c>
       <c r="B49" t="s">
@@ -1813,9 +1717,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50">
-        <f>--_xlfn.TEXTBEFORE(B50,".")</f>
+        <f t="shared" si="1"/>
         <v>591</v>
       </c>
       <c r="B50" t="s">
@@ -1828,9 +1732,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51">
-        <f>--_xlfn.TEXTBEFORE(B51,".")</f>
+        <f t="shared" si="1"/>
         <v>592</v>
       </c>
       <c r="B51" t="s">
@@ -1843,9 +1747,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52">
-        <f>--_xlfn.TEXTBEFORE(B52,".")</f>
+        <f t="shared" si="1"/>
         <v>593</v>
       </c>
       <c r="B52" t="s">
@@ -1858,9 +1762,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53">
-        <f>--_xlfn.TEXTBEFORE(B53,".")</f>
+        <f t="shared" si="1"/>
         <v>594</v>
       </c>
       <c r="B53" t="s">
@@ -1873,9 +1777,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54">
-        <f>--_xlfn.TEXTBEFORE(B54,".")</f>
+        <f t="shared" si="1"/>
         <v>607</v>
       </c>
       <c r="B54" t="s">
@@ -1888,9 +1792,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55">
-        <f>--_xlfn.TEXTBEFORE(B55,".")</f>
+        <f t="shared" si="1"/>
         <v>615</v>
       </c>
       <c r="B55" t="s">
@@ -1903,27 +1807,24 @@
         <v>179</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56">
-        <f>--_xlfn.TEXTBEFORE(B56,".")</f>
+        <f t="shared" si="1"/>
         <v>628</v>
       </c>
       <c r="B56" t="s">
         <v>80</v>
       </c>
       <c r="C56" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D56" t="s">
         <v>179</v>
       </c>
-      <c r="E56" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57">
-        <f>--_xlfn.TEXTBEFORE(B57,".")</f>
+        <f t="shared" si="1"/>
         <v>636</v>
       </c>
       <c r="B57" t="s">
@@ -1936,9 +1837,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58">
-        <f>--_xlfn.TEXTBEFORE(B58,".")</f>
+        <f t="shared" si="1"/>
         <v>637</v>
       </c>
       <c r="B58" t="s">
@@ -1951,9 +1852,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59">
-        <f>--_xlfn.TEXTBEFORE(B59,".")</f>
+        <f t="shared" si="1"/>
         <v>638</v>
       </c>
       <c r="B59" t="s">
@@ -1966,9 +1867,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60">
-        <f>--_xlfn.TEXTBEFORE(B60,".")</f>
+        <f t="shared" si="1"/>
         <v>639</v>
       </c>
       <c r="B60" t="s">
@@ -1981,9 +1882,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61">
-        <f>--_xlfn.TEXTBEFORE(B61,".")</f>
+        <f t="shared" si="1"/>
         <v>642</v>
       </c>
       <c r="B61" t="s">
@@ -1996,9 +1897,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62">
-        <f>--_xlfn.TEXTBEFORE(B62,".")</f>
+        <f t="shared" si="1"/>
         <v>643</v>
       </c>
       <c r="B62" t="s">
@@ -2011,9 +1912,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63">
-        <f>--_xlfn.TEXTBEFORE(B63,".")</f>
+        <f t="shared" si="1"/>
         <v>644</v>
       </c>
       <c r="B63" t="s">
@@ -2026,9 +1927,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64">
-        <f>--_xlfn.TEXTBEFORE(B64,".")</f>
+        <f t="shared" si="1"/>
         <v>645</v>
       </c>
       <c r="B64" t="s">
@@ -2041,9 +1942,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65">
-        <f>--_xlfn.TEXTBEFORE(B65,".")</f>
+        <f t="shared" si="1"/>
         <v>657</v>
       </c>
       <c r="B65" t="s">
@@ -2056,9 +1957,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66">
-        <f>--_xlfn.TEXTBEFORE(B66,".")</f>
+        <f t="shared" ref="A66:A97" si="2">--_xlfn.TEXTBEFORE(B66,".")</f>
         <v>659</v>
       </c>
       <c r="B66" t="s">
@@ -2071,9 +1972,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67">
-        <f>--_xlfn.TEXTBEFORE(B67,".")</f>
+        <f t="shared" si="2"/>
         <v>665</v>
       </c>
       <c r="B67" t="s">
@@ -2086,9 +1987,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68">
-        <f>--_xlfn.TEXTBEFORE(B68,".")</f>
+        <f t="shared" si="2"/>
         <v>666</v>
       </c>
       <c r="B68" t="s">
@@ -2101,9 +2002,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69">
-        <f>--_xlfn.TEXTBEFORE(B69,".")</f>
+        <f t="shared" si="2"/>
         <v>669</v>
       </c>
       <c r="B69" t="s">
@@ -2116,9 +2017,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70">
-        <f>--_xlfn.TEXTBEFORE(B70,".")</f>
+        <f t="shared" si="2"/>
         <v>670</v>
       </c>
       <c r="B70" t="s">
@@ -2131,9 +2032,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71">
-        <f>--_xlfn.TEXTBEFORE(B71,".")</f>
+        <f t="shared" si="2"/>
         <v>672</v>
       </c>
       <c r="B71" t="s">
@@ -2146,9 +2047,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72">
-        <f>--_xlfn.TEXTBEFORE(B72,".")</f>
+        <f t="shared" si="2"/>
         <v>673</v>
       </c>
       <c r="B72" t="s">
@@ -2161,9 +2062,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73">
-        <f>--_xlfn.TEXTBEFORE(B73,".")</f>
+        <f t="shared" si="2"/>
         <v>674</v>
       </c>
       <c r="B73" t="s">
@@ -2176,9 +2077,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74">
-        <f>--_xlfn.TEXTBEFORE(B74,".")</f>
+        <f t="shared" si="2"/>
         <v>675</v>
       </c>
       <c r="B74" t="s">
@@ -2191,9 +2092,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75">
-        <f>--_xlfn.TEXTBEFORE(B75,".")</f>
+        <f t="shared" si="2"/>
         <v>676</v>
       </c>
       <c r="B75" t="s">
@@ -2206,27 +2107,24 @@
         <v>179</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76">
-        <f>--_xlfn.TEXTBEFORE(B76,".")</f>
+        <f t="shared" si="2"/>
         <v>680</v>
       </c>
       <c r="B76" t="s">
         <v>101</v>
       </c>
       <c r="C76" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="D76" t="s">
-        <v>188</v>
-      </c>
-      <c r="E76" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77">
-        <f>--_xlfn.TEXTBEFORE(B77,".")</f>
+        <f t="shared" si="2"/>
         <v>681</v>
       </c>
       <c r="B77" t="s">
@@ -2239,45 +2137,39 @@
         <v>179</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78">
-        <f>--_xlfn.TEXTBEFORE(B78,".")</f>
+        <f t="shared" si="2"/>
         <v>689</v>
       </c>
       <c r="B78" t="s">
         <v>103</v>
       </c>
       <c r="C78" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="D78" t="s">
-        <v>188</v>
-      </c>
-      <c r="E78" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79">
-        <f>--_xlfn.TEXTBEFORE(B79,".")</f>
+        <f t="shared" si="2"/>
         <v>694</v>
       </c>
       <c r="B79" t="s">
         <v>104</v>
       </c>
       <c r="C79" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D79" t="s">
-        <v>182</v>
-      </c>
-      <c r="E79" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80">
-        <f>--_xlfn.TEXTBEFORE(B80,".")</f>
+        <f t="shared" si="2"/>
         <v>726</v>
       </c>
       <c r="B80" t="s">
@@ -2292,7 +2184,7 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81">
-        <f>--_xlfn.TEXTBEFORE(B81,".")</f>
+        <f t="shared" si="2"/>
         <v>727</v>
       </c>
       <c r="B81" t="s">
@@ -2307,7 +2199,7 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82">
-        <f>--_xlfn.TEXTBEFORE(B82,".")</f>
+        <f t="shared" si="2"/>
         <v>728</v>
       </c>
       <c r="B82" t="s">
@@ -2322,7 +2214,7 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83">
-        <f>--_xlfn.TEXTBEFORE(B83,".")</f>
+        <f t="shared" si="2"/>
         <v>730</v>
       </c>
       <c r="B83" t="s">
@@ -2337,7 +2229,7 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84">
-        <f>--_xlfn.TEXTBEFORE(B84,".")</f>
+        <f t="shared" si="2"/>
         <v>731</v>
       </c>
       <c r="B84" t="s">
@@ -2352,7 +2244,7 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85">
-        <f>--_xlfn.TEXTBEFORE(B85,".")</f>
+        <f t="shared" si="2"/>
         <v>732</v>
       </c>
       <c r="B85" t="s">
@@ -2367,7 +2259,7 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86">
-        <f>--_xlfn.TEXTBEFORE(B86,".")</f>
+        <f t="shared" si="2"/>
         <v>733</v>
       </c>
       <c r="B86" t="s">
@@ -2382,7 +2274,7 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87">
-        <f>--_xlfn.TEXTBEFORE(B87,".")</f>
+        <f t="shared" si="2"/>
         <v>734</v>
       </c>
       <c r="B87" t="s">
@@ -2397,7 +2289,7 @@
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88">
-        <f>--_xlfn.TEXTBEFORE(B88,".")</f>
+        <f t="shared" si="2"/>
         <v>737</v>
       </c>
       <c r="B88" t="s">
@@ -2412,7 +2304,7 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89">
-        <f>--_xlfn.TEXTBEFORE(B89,".")</f>
+        <f t="shared" si="2"/>
         <v>740</v>
       </c>
       <c r="B89" t="s">
@@ -2427,7 +2319,7 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90">
-        <f>--_xlfn.TEXTBEFORE(B90,".")</f>
+        <f t="shared" si="2"/>
         <v>741</v>
       </c>
       <c r="B90" t="s">
@@ -2442,7 +2334,7 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91">
-        <f>--_xlfn.TEXTBEFORE(B91,".")</f>
+        <f t="shared" si="2"/>
         <v>743</v>
       </c>
       <c r="B91" t="s">
@@ -2457,7 +2349,7 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92">
-        <f>--_xlfn.TEXTBEFORE(B92,".")</f>
+        <f t="shared" si="2"/>
         <v>748</v>
       </c>
       <c r="B92" t="s">
@@ -2472,7 +2364,7 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93">
-        <f>--_xlfn.TEXTBEFORE(B93,".")</f>
+        <f t="shared" si="2"/>
         <v>751</v>
       </c>
       <c r="B93" t="s">
@@ -2487,7 +2379,7 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94">
-        <f>--_xlfn.TEXTBEFORE(B94,".")</f>
+        <f t="shared" si="2"/>
         <v>759</v>
       </c>
       <c r="B94" t="s">
@@ -2502,7 +2394,7 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95">
-        <f>--_xlfn.TEXTBEFORE(B95,".")</f>
+        <f t="shared" si="2"/>
         <v>762</v>
       </c>
       <c r="B95" t="s">
@@ -2517,7 +2409,7 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96">
-        <f>--_xlfn.TEXTBEFORE(B96,".")</f>
+        <f t="shared" si="2"/>
         <v>772</v>
       </c>
       <c r="B96" t="s">
@@ -2530,9 +2422,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97">
-        <f>--_xlfn.TEXTBEFORE(B97,".")</f>
+        <f t="shared" si="2"/>
         <v>782</v>
       </c>
       <c r="B97" t="s">
@@ -2545,9 +2437,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98">
-        <f>--_xlfn.TEXTBEFORE(B98,".")</f>
+        <f t="shared" ref="A98:A129" si="3">--_xlfn.TEXTBEFORE(B98,".")</f>
         <v>783</v>
       </c>
       <c r="B98" t="s">
@@ -2560,9 +2452,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99">
-        <f>--_xlfn.TEXTBEFORE(B99,".")</f>
+        <f t="shared" si="3"/>
         <v>784</v>
       </c>
       <c r="B99" t="s">
@@ -2575,9 +2467,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100">
-        <f>--_xlfn.TEXTBEFORE(B100,".")</f>
+        <f t="shared" si="3"/>
         <v>790</v>
       </c>
       <c r="B100" t="s">
@@ -2590,9 +2482,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101">
-        <f>--_xlfn.TEXTBEFORE(B101,".")</f>
+        <f t="shared" si="3"/>
         <v>807</v>
       </c>
       <c r="B101" t="s">
@@ -2605,63 +2497,54 @@
         <v>179</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102">
-        <f>--_xlfn.TEXTBEFORE(B102,".")</f>
+        <f t="shared" si="3"/>
         <v>808</v>
       </c>
       <c r="B102" t="s">
         <v>128</v>
       </c>
       <c r="C102" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D102" t="s">
-        <v>182</v>
-      </c>
-      <c r="E102" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103">
-        <f>--_xlfn.TEXTBEFORE(B103,".")</f>
+        <f t="shared" si="3"/>
         <v>810</v>
       </c>
       <c r="B103" t="s">
         <v>129</v>
       </c>
       <c r="C103" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D103" t="s">
-        <v>182</v>
-      </c>
-      <c r="E103" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104">
-        <f>--_xlfn.TEXTBEFORE(B104,".")</f>
+        <f t="shared" si="3"/>
         <v>828</v>
       </c>
       <c r="B104" t="s">
         <v>130</v>
       </c>
       <c r="C104" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D104" t="s">
-        <v>182</v>
-      </c>
-      <c r="E104" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105">
-        <f>--_xlfn.TEXTBEFORE(B105,".")</f>
+        <f t="shared" si="3"/>
         <v>842</v>
       </c>
       <c r="B105" t="s">
@@ -2674,9 +2557,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106">
-        <f>--_xlfn.TEXTBEFORE(B106,".")</f>
+        <f t="shared" si="3"/>
         <v>843</v>
       </c>
       <c r="B106" t="s">
@@ -2689,9 +2572,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107">
-        <f>--_xlfn.TEXTBEFORE(B107,".")</f>
+        <f t="shared" si="3"/>
         <v>847</v>
       </c>
       <c r="B107" t="s">
@@ -2704,9 +2587,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108">
-        <f>--_xlfn.TEXTBEFORE(B108,".")</f>
+        <f t="shared" si="3"/>
         <v>851</v>
       </c>
       <c r="B108" t="s">
@@ -2719,9 +2602,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109">
-        <f>--_xlfn.TEXTBEFORE(B109,".")</f>
+        <f t="shared" si="3"/>
         <v>852</v>
       </c>
       <c r="B109" t="s">
@@ -2734,9 +2617,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110">
-        <f>--_xlfn.TEXTBEFORE(B110,".")</f>
+        <f t="shared" si="3"/>
         <v>857</v>
       </c>
       <c r="B110" t="s">
@@ -2749,9 +2632,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111">
-        <f>--_xlfn.TEXTBEFORE(B111,".")</f>
+        <f t="shared" si="3"/>
         <v>858</v>
       </c>
       <c r="B111" t="s">
@@ -2764,9 +2647,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112">
-        <f>--_xlfn.TEXTBEFORE(B112,".")</f>
+        <f t="shared" si="3"/>
         <v>865</v>
       </c>
       <c r="B112" t="s">
@@ -2781,7 +2664,7 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113">
-        <f>--_xlfn.TEXTBEFORE(B113,".")</f>
+        <f t="shared" si="3"/>
         <v>866</v>
       </c>
       <c r="B113" t="s">
@@ -2796,7 +2679,7 @@
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114">
-        <f>--_xlfn.TEXTBEFORE(B114,".")</f>
+        <f t="shared" si="3"/>
         <v>867</v>
       </c>
       <c r="B114" t="s">
@@ -2811,7 +2694,7 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115">
-        <f>--_xlfn.TEXTBEFORE(B115,".")</f>
+        <f t="shared" si="3"/>
         <v>868</v>
       </c>
       <c r="B115" t="s">
@@ -2826,7 +2709,7 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116">
-        <f>--_xlfn.TEXTBEFORE(B116,".")</f>
+        <f t="shared" si="3"/>
         <v>869</v>
       </c>
       <c r="B116" t="s">
@@ -2841,7 +2724,7 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117">
-        <f>--_xlfn.TEXTBEFORE(B117,".")</f>
+        <f t="shared" si="3"/>
         <v>870</v>
       </c>
       <c r="B117" t="s">
@@ -2856,7 +2739,7 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118">
-        <f>--_xlfn.TEXTBEFORE(B118,".")</f>
+        <f t="shared" si="3"/>
         <v>874</v>
       </c>
       <c r="B118" t="s">
@@ -2871,7 +2754,7 @@
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119">
-        <f>--_xlfn.TEXTBEFORE(B119,".")</f>
+        <f t="shared" si="3"/>
         <v>876</v>
       </c>
       <c r="B119" t="s">
@@ -2886,7 +2769,7 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120">
-        <f>--_xlfn.TEXTBEFORE(B120,".")</f>
+        <f t="shared" si="3"/>
         <v>878</v>
       </c>
       <c r="B120" t="s">
@@ -2901,7 +2784,7 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121">
-        <f>--_xlfn.TEXTBEFORE(B121,".")</f>
+        <f t="shared" si="3"/>
         <v>903</v>
       </c>
       <c r="B121" t="s">
@@ -2916,7 +2799,7 @@
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122">
-        <f>--_xlfn.TEXTBEFORE(B122,".")</f>
+        <f t="shared" si="3"/>
         <v>908</v>
       </c>
       <c r="B122" t="s">
@@ -2931,7 +2814,7 @@
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123">
-        <f>--_xlfn.TEXTBEFORE(B123,".")</f>
+        <f t="shared" si="3"/>
         <v>909</v>
       </c>
       <c r="B123" t="s">
@@ -2946,7 +2829,7 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124">
-        <f>--_xlfn.TEXTBEFORE(B124,".")</f>
+        <f t="shared" si="3"/>
         <v>911</v>
       </c>
       <c r="B124" t="s">
@@ -2961,7 +2844,7 @@
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125">
-        <f>--_xlfn.TEXTBEFORE(B125,".")</f>
+        <f t="shared" si="3"/>
         <v>914</v>
       </c>
       <c r="B125" t="s">
@@ -2976,7 +2859,7 @@
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126">
-        <f>--_xlfn.TEXTBEFORE(B126,".")</f>
+        <f t="shared" si="3"/>
         <v>916</v>
       </c>
       <c r="B126" t="s">
@@ -2991,7 +2874,7 @@
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127">
-        <f>--_xlfn.TEXTBEFORE(B127,".")</f>
+        <f t="shared" si="3"/>
         <v>917</v>
       </c>
       <c r="B127" t="s">
@@ -3006,7 +2889,7 @@
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128">
-        <f>--_xlfn.TEXTBEFORE(B128,".")</f>
+        <f t="shared" si="3"/>
         <v>918</v>
       </c>
       <c r="B128" t="s">
@@ -3019,9 +2902,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129">
-        <f>--_xlfn.TEXTBEFORE(B129,".")</f>
+        <f t="shared" si="3"/>
         <v>922</v>
       </c>
       <c r="B129" t="s">
@@ -3034,9 +2917,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130">
-        <f>--_xlfn.TEXTBEFORE(B130,".")</f>
+        <f t="shared" ref="A130:A161" si="4">--_xlfn.TEXTBEFORE(B130,".")</f>
         <v>923</v>
       </c>
       <c r="B130" t="s">
@@ -3049,9 +2932,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131">
-        <f>--_xlfn.TEXTBEFORE(B131,".")</f>
+        <f t="shared" si="4"/>
         <v>937</v>
       </c>
       <c r="B131" t="s">
@@ -3064,9 +2947,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132">
-        <f>--_xlfn.TEXTBEFORE(B132,".")</f>
+        <f t="shared" si="4"/>
         <v>940</v>
       </c>
       <c r="B132" t="s">
@@ -3079,9 +2962,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133">
-        <f>--_xlfn.TEXTBEFORE(B133,".")</f>
+        <f t="shared" si="4"/>
         <v>941</v>
       </c>
       <c r="B133" t="s">
@@ -3094,9 +2977,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134">
-        <f>--_xlfn.TEXTBEFORE(B134,".")</f>
+        <f t="shared" si="4"/>
         <v>942</v>
       </c>
       <c r="B134" t="s">
@@ -3109,9 +2992,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135">
-        <f>--_xlfn.TEXTBEFORE(B135,".")</f>
+        <f t="shared" si="4"/>
         <v>949</v>
       </c>
       <c r="B135" t="s">
@@ -3124,9 +3007,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136">
-        <f>--_xlfn.TEXTBEFORE(B136,".")</f>
+        <f t="shared" si="4"/>
         <v>951</v>
       </c>
       <c r="B136" t="s">
@@ -3139,27 +3022,24 @@
         <v>179</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137">
-        <f>--_xlfn.TEXTBEFORE(B137,".")</f>
+        <f t="shared" si="4"/>
         <v>954</v>
       </c>
       <c r="B137" t="s">
         <v>165</v>
       </c>
       <c r="C137" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D137" t="s">
-        <v>182</v>
-      </c>
-      <c r="E137" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138">
-        <f>--_xlfn.TEXTBEFORE(B138,".")</f>
+        <f t="shared" si="4"/>
         <v>955</v>
       </c>
       <c r="B138" t="s">
@@ -3172,9 +3052,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139">
-        <f>--_xlfn.TEXTBEFORE(B139,".")</f>
+        <f t="shared" si="4"/>
         <v>958</v>
       </c>
       <c r="B139" t="s">
@@ -3187,9 +3067,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140">
-        <f>--_xlfn.TEXTBEFORE(B140,".")</f>
+        <f t="shared" si="4"/>
         <v>972</v>
       </c>
       <c r="B140" t="s">
@@ -3202,9 +3082,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141">
-        <f>--_xlfn.TEXTBEFORE(B141,".")</f>
+        <f t="shared" si="4"/>
         <v>973</v>
       </c>
       <c r="B141" t="s">
@@ -3217,9 +3097,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142">
-        <f>--_xlfn.TEXTBEFORE(B142,".")</f>
+        <f t="shared" si="4"/>
         <v>974</v>
       </c>
       <c r="B142" t="s">
@@ -3232,9 +3112,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143">
-        <f>--_xlfn.TEXTBEFORE(B143,".")</f>
+        <f t="shared" si="4"/>
         <v>987</v>
       </c>
       <c r="B143" t="s">
@@ -3247,9 +3127,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144">
-        <f>--_xlfn.TEXTBEFORE(B144,".")</f>
+        <f t="shared" si="4"/>
         <v>1000</v>
       </c>
       <c r="B144" t="s">
@@ -3262,9 +3142,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145">
-        <f>--_xlfn.TEXTBEFORE(B145,".")</f>
+        <f t="shared" si="4"/>
         <v>1002</v>
       </c>
       <c r="B145" t="s">
@@ -3277,9 +3157,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146">
-        <f>--_xlfn.TEXTBEFORE(B146,".")</f>
+        <f t="shared" si="4"/>
         <v>1003</v>
       </c>
       <c r="B146" t="s">
@@ -3292,27 +3172,24 @@
         <v>179</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147">
-        <f>--_xlfn.TEXTBEFORE(B147,".")</f>
+        <f t="shared" si="4"/>
         <v>1004</v>
       </c>
       <c r="B147" t="s">
         <v>3</v>
       </c>
       <c r="C147" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D147" t="s">
-        <v>182</v>
-      </c>
-      <c r="E147" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148">
-        <f>--_xlfn.TEXTBEFORE(B148,".")</f>
+        <f t="shared" si="4"/>
         <v>1005</v>
       </c>
       <c r="B148" t="s">
@@ -3325,27 +3202,24 @@
         <v>179</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149">
-        <f>--_xlfn.TEXTBEFORE(B149,".")</f>
+        <f t="shared" si="4"/>
         <v>1007</v>
       </c>
       <c r="B149" t="s">
         <v>5</v>
       </c>
       <c r="C149" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D149" t="s">
-        <v>182</v>
-      </c>
-      <c r="E149" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150">
-        <f>--_xlfn.TEXTBEFORE(B150,".")</f>
+        <f t="shared" si="4"/>
         <v>1008</v>
       </c>
       <c r="B150" t="s">
@@ -3358,9 +3232,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151">
-        <f>--_xlfn.TEXTBEFORE(B151,".")</f>
+        <f t="shared" si="4"/>
         <v>1018</v>
       </c>
       <c r="B151" t="s">
@@ -3373,9 +3247,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152">
-        <f>--_xlfn.TEXTBEFORE(B152,".")</f>
+        <f t="shared" si="4"/>
         <v>1022</v>
       </c>
       <c r="B152" t="s">
@@ -3388,9 +3262,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153">
-        <f>--_xlfn.TEXTBEFORE(B153,".")</f>
+        <f t="shared" si="4"/>
         <v>1023</v>
       </c>
       <c r="B153" t="s">
@@ -3403,9 +3277,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154">
-        <f>--_xlfn.TEXTBEFORE(B154,".")</f>
+        <f t="shared" si="4"/>
         <v>1024</v>
       </c>
       <c r="B154" t="s">
@@ -3418,9 +3292,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155">
-        <f>--_xlfn.TEXTBEFORE(B155,".")</f>
+        <f t="shared" si="4"/>
         <v>1027</v>
       </c>
       <c r="B155" t="s">
@@ -3433,9 +3307,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156">
-        <f>--_xlfn.TEXTBEFORE(B156,".")</f>
+        <f t="shared" si="4"/>
         <v>1028</v>
       </c>
       <c r="B156" t="s">
@@ -3448,9 +3322,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157">
-        <f>--_xlfn.TEXTBEFORE(B157,".")</f>
+        <f t="shared" si="4"/>
         <v>1029</v>
       </c>
       <c r="B157" t="s">
@@ -3463,9 +3337,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158">
-        <f>--_xlfn.TEXTBEFORE(B158,".")</f>
+        <f t="shared" si="4"/>
         <v>1030</v>
       </c>
       <c r="B158" t="s">
@@ -3478,9 +3352,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159">
-        <f>--_xlfn.TEXTBEFORE(B159,".")</f>
+        <f t="shared" si="4"/>
         <v>1031</v>
       </c>
       <c r="B159" t="s">
@@ -3493,9 +3367,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160">
-        <f>--_xlfn.TEXTBEFORE(B160,".")</f>
+        <f t="shared" si="4"/>
         <v>1032</v>
       </c>
       <c r="B160" t="s">
@@ -3508,9 +3382,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161">
-        <f>--_xlfn.TEXTBEFORE(B161,".")</f>
+        <f t="shared" si="4"/>
         <v>1033</v>
       </c>
       <c r="B161" t="s">
@@ -3523,9 +3397,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162">
-        <f>--_xlfn.TEXTBEFORE(B162,".")</f>
+        <f t="shared" ref="A162:A175" si="5">--_xlfn.TEXTBEFORE(B162,".")</f>
         <v>1034</v>
       </c>
       <c r="B162" t="s">
@@ -3538,9 +3412,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163">
-        <f>--_xlfn.TEXTBEFORE(B163,".")</f>
+        <f t="shared" si="5"/>
         <v>1035</v>
       </c>
       <c r="B163" t="s">
@@ -3553,9 +3427,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164">
-        <f>--_xlfn.TEXTBEFORE(B164,".")</f>
+        <f t="shared" si="5"/>
         <v>1044</v>
       </c>
       <c r="B164" t="s">
@@ -3568,9 +3442,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165">
-        <f>--_xlfn.TEXTBEFORE(B165,".")</f>
+        <f t="shared" si="5"/>
         <v>1048</v>
       </c>
       <c r="B165" t="s">
@@ -3583,9 +3457,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166">
-        <f>--_xlfn.TEXTBEFORE(B166,".")</f>
+        <f t="shared" si="5"/>
         <v>1051</v>
       </c>
       <c r="B166" t="s">
@@ -3598,9 +3472,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167">
-        <f>--_xlfn.TEXTBEFORE(B167,".")</f>
+        <f t="shared" si="5"/>
         <v>1052</v>
       </c>
       <c r="B167" t="s">
@@ -3613,9 +3487,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168">
-        <f>--_xlfn.TEXTBEFORE(B168,".")</f>
+        <f t="shared" si="5"/>
         <v>1055</v>
       </c>
       <c r="B168" t="s">
@@ -3628,9 +3502,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169">
-        <f>--_xlfn.TEXTBEFORE(B169,".")</f>
+        <f t="shared" si="5"/>
         <v>1056</v>
       </c>
       <c r="B169" t="s">
@@ -3643,9 +3517,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170">
-        <f>--_xlfn.TEXTBEFORE(B170,".")</f>
+        <f t="shared" si="5"/>
         <v>1058</v>
       </c>
       <c r="B170" t="s">
@@ -3658,9 +3532,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171">
-        <f>--_xlfn.TEXTBEFORE(B171,".")</f>
+        <f t="shared" si="5"/>
         <v>1060</v>
       </c>
       <c r="B171" t="s">
@@ -3673,9 +3547,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172">
-        <f>--_xlfn.TEXTBEFORE(B172,".")</f>
+        <f t="shared" si="5"/>
         <v>1064</v>
       </c>
       <c r="B172" t="s">
@@ -3688,9 +3562,9 @@
         <v>179</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173">
-        <f>--_xlfn.TEXTBEFORE(B173,".")</f>
+        <f t="shared" si="5"/>
         <v>1071</v>
       </c>
       <c r="B173" t="s">
@@ -3703,27 +3577,24 @@
         <v>179</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174">
-        <f>--_xlfn.TEXTBEFORE(B174,".")</f>
+        <f t="shared" si="5"/>
         <v>1072</v>
       </c>
       <c r="B174" t="s">
         <v>31</v>
       </c>
       <c r="C174" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D174" t="s">
-        <v>182</v>
-      </c>
-      <c r="E174" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175">
-        <f>--_xlfn.TEXTBEFORE(B175,".")</f>
+        <f t="shared" si="5"/>
         <v>1075</v>
       </c>
       <c r="B175" t="s">

</xml_diff>